<commit_message>
Day 11 - Full pipeline assembled: PDF to Excel in 4 clean functions
</commit_message>
<xml_diff>
--- a/invoices_output.xlsx
+++ b/invoices_output.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Invoices" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,10 +449,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1253888565</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1253888565</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -475,10 +473,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1253642565</t>
-        </is>
+      <c r="A3" t="n">
+        <v>1253642565</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -501,10 +497,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1253743874</t>
-        </is>
+      <c r="A4" t="n">
+        <v>1253743874</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -524,6 +518,32 @@
       </c>
       <c r="F4" t="n">
         <v>454.49</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1253888565</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>27.04.2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SYSCO France SAS</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>526.47</v>
+      </c>
+      <c r="E5" t="n">
+        <v>28.96</v>
+      </c>
+      <c r="F5" t="n">
+        <v>555.4299999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Day 12 - Streamlit interface complete
</commit_message>
<xml_diff>
--- a/invoices_output.xlsx
+++ b/invoices_output.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,10 +521,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1253888565</t>
-        </is>
+      <c r="A5" t="n">
+        <v>1253888565</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -543,6 +541,32 @@
         <v>28.96</v>
       </c>
       <c r="F5" t="n">
+        <v>555.4299999999999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1253888565</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>27.04.2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SYSCO France SAS</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>526.47</v>
+      </c>
+      <c r="E6" t="n">
+        <v>28.96</v>
+      </c>
+      <c r="F6" t="n">
         <v>555.4299999999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Day 13 - Hotel Invoice Extractor complete
</commit_message>
<xml_diff>
--- a/invoices_output.xlsx
+++ b/invoices_output.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,10 +545,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1253888565</t>
-        </is>
+      <c r="A6" t="n">
+        <v>1253888565</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -567,6 +565,32 @@
         <v>28.96</v>
       </c>
       <c r="F6" t="n">
+        <v>555.4299999999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1253888565</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>27.04.2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SYSCO France SAS</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>526.47</v>
+      </c>
+      <c r="E7" t="n">
+        <v>28.96</v>
+      </c>
+      <c r="F7" t="n">
         <v>555.4299999999999</v>
       </c>
     </row>

</xml_diff>